<commit_message>
Publish plain-language capital plan assets
</commit_message>
<xml_diff>
--- a/assets/MUD2-Capital-Plan-analysis.xlsx
+++ b/assets/MUD2-Capital-Plan-analysis.xlsx
@@ -1412,7 +1412,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Capital Base Fee as proposed ($100/connection)</t>
+          <t>Capital Base Fee as proposed ($100 per home/account)</t>
         </is>
       </c>
       <c r="B4" s="8" t="n">
@@ -1441,7 +1441,7 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Cash-fund the whole plan from a fee</t>
+          <t>Pay cash for the whole plan via a fee</t>
         </is>
       </c>
       <c r="B5" s="10" t="n">
@@ -1470,7 +1470,7 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Debt-fund the whole plan (25 yr @ 4.25%)</t>
+          <t>Bond the whole plan (25 yr @ 4.25%)</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
@@ -1499,7 +1499,7 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Match funding to asset life (recommended)</t>
+          <t>Split: repairs from rates, equipment on bonds (recommended)</t>
         </is>
       </c>
       <c r="B7" s="10" t="n">
@@ -1600,7 +1600,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Flat fee per connection</t>
+          <t>Flat fee per home/account</t>
         </is>
       </c>
       <c r="B4" s="8" t="n">
@@ -1624,7 +1624,7 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Debt service tax — commercial 20% of value</t>
+          <t>Bond-repayment tax — commercial 20% of value</t>
         </is>
       </c>
       <c r="B5" s="10" t="n">
@@ -1648,7 +1648,7 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Debt service tax — commercial 35% of value</t>
+          <t>Bond-repayment tax — commercial 35% of value</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
@@ -1672,7 +1672,7 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Debt service tax — commercial 48% of value</t>
+          <t>Bond-repayment tax — commercial 48% of value</t>
         </is>
       </c>
       <c r="B7" s="10" t="n">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Debt service tax / month</t>
+          <t>Bond-repayment tax / month</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -1966,7 +1966,7 @@
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>Debt service tax rate $0.138167 per $100 of taxable value. Break-even at $868,517. The after-deduction column applies only to households that itemise and sit under the 2026 SALT cap of $40,400; most take the standard deduction and capture none of it.</t>
+          <t>Bond-repayment tax rate $0.138167 per $100 of taxable value. Break-even at $868,517. The after-deduction column applies only to households that itemise and sit under the 2026 SALT cap of $40,400; most take the standard deduction and capture none of it.</t>
         </is>
       </c>
     </row>

</xml_diff>